<commit_message>
Update student LeetCode IDs
</commit_message>
<xml_diff>
--- a/students/leetcode_Links.xlsx
+++ b/students/leetcode_Links.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KALAI\Documents\Leetcode-Automation\students\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53781062-DB08-455C-9ADA-FE211AE56839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C93148F3-93CF-4071-BF49-6F559B87842D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1572" windowWidth="23040" windowHeight="11388" xr2:uid="{A1D85D54-F45A-40AC-9A85-717C16392CF8}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{A1D85D54-F45A-40AC-9A85-717C16392CF8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
   <si>
     <t>S.No</t>
   </si>
@@ -98,9 +98,6 @@
     <t>CHARAN SAI PATHAPATHI</t>
   </si>
   <si>
-    <t>CHARAN_08</t>
-  </si>
-  <si>
     <t>CHERUKURU THANUJA</t>
   </si>
   <si>
@@ -188,9 +185,6 @@
     <t>LOHITH D</t>
   </si>
   <si>
-    <t>lohith_d</t>
-  </si>
-  <si>
     <t>M JESIN MILESH</t>
   </si>
   <si>
@@ -257,9 +251,6 @@
     <t>PRAVEEN KUMAR.S</t>
   </si>
   <si>
-    <t>S. Praveen Kumar</t>
-  </si>
-  <si>
     <t>PRIYA G</t>
   </si>
   <si>
@@ -320,9 +311,6 @@
     <t>SURENDHAR B</t>
   </si>
   <si>
-    <t>Surendar777</t>
-  </si>
-  <si>
     <t>THIRUSELVEN P</t>
   </si>
   <si>
@@ -353,9 +341,6 @@
     <t>https://leetcode.com/u/BOOPESH_SB/</t>
   </si>
   <si>
-    <t>https://leetcode.com/u/CHARAN_08/</t>
-  </si>
-  <si>
     <t>https://leetcode.com/u/thanuja_cherukuru/</t>
   </si>
   <si>
@@ -404,9 +389,6 @@
     <t>https://leetcode.com/u/liyasali/</t>
   </si>
   <si>
-    <t>https://leetcode.com/u/lohith_d/</t>
-  </si>
-  <si>
     <t>https://leetcode.com/u/manu-25/</t>
   </si>
   <si>
@@ -446,9 +428,6 @@
     <t>https://leetcode.com/u/Rahul0218/</t>
   </si>
   <si>
-    <t>https://leetcode.com/u/praveen-s-kumar/</t>
-  </si>
-  <si>
     <t>https://leetcode.com/u/subhash_chowdary09/</t>
   </si>
   <si>
@@ -467,9 +446,6 @@
     <t>https://leetcode.com/u/SUJITHKUMAR1234/</t>
   </si>
   <si>
-    <t>https://leetcode.com/u/Surendar777/</t>
-  </si>
-  <si>
     <t>https://leetcode.com/u/yuthish_29/</t>
   </si>
   <si>
@@ -483,6 +459,33 @@
   </si>
   <si>
     <t>IroXEV3ekA</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/u/YSLGIbeAtA/</t>
+  </si>
+  <si>
+    <t>YSLGIbeAtA</t>
+  </si>
+  <si>
+    <t>lohith_yadav</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/u/lohith_yadav/</t>
+  </si>
+  <si>
+    <t>l0RNz5nLnd</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/u/l0RNz5nLnd/</t>
+  </si>
+  <si>
+    <t>HRamamoorthy</t>
+  </si>
+  <si>
+    <t>surendhar777</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/u/surendhar777/</t>
   </si>
 </sst>
 </file>
@@ -706,10 +709,10 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1069,7 +1072,7 @@
         <v>3</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1086,7 +1089,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1103,7 +1106,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1119,8 +1122,8 @@
       <c r="D6" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="12" t="s">
-        <v>101</v>
+      <c r="E6" s="11" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1136,8 +1139,8 @@
       <c r="D7" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="12" t="s">
-        <v>102</v>
+      <c r="E7" s="11" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1154,7 +1157,7 @@
         <v>13</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1171,7 +1174,7 @@
         <v>15</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1187,11 +1190,11 @@
       <c r="D10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="12" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E10" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>8</v>
       </c>
@@ -1202,10 +1205,10 @@
         <v>18</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>104</v>
+        <v>141</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1216,13 +1219,13 @@
         <v>111424149009</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>105</v>
+      <c r="E12" s="11" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1233,13 +1236,13 @@
         <v>111424149010</v>
       </c>
       <c r="C13" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="9" t="s">
-        <v>23</v>
-      </c>
       <c r="E13" s="10" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1250,13 +1253,13 @@
         <v>111424149011</v>
       </c>
       <c r="C14" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="9" t="s">
-        <v>25</v>
-      </c>
       <c r="E14" s="10" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
@@ -1267,13 +1270,13 @@
         <v>111424149012</v>
       </c>
       <c r="C15" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="9" t="s">
-        <v>27</v>
-      </c>
       <c r="E15" s="10" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1284,13 +1287,13 @@
         <v>111424149007</v>
       </c>
       <c r="C16" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>29</v>
-      </c>
       <c r="E16" s="10" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1301,13 +1304,13 @@
         <v>111424149014</v>
       </c>
       <c r="C17" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="E17" s="12" t="s">
-        <v>112</v>
+      <c r="E17" s="11" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1318,13 +1321,13 @@
         <v>111424149015</v>
       </c>
       <c r="C18" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>33</v>
-      </c>
       <c r="E18" s="10" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
@@ -1335,13 +1338,13 @@
         <v>111424149016</v>
       </c>
       <c r="C19" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="9" t="s">
-        <v>35</v>
-      </c>
       <c r="E19" s="10" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1352,13 +1355,13 @@
         <v>111424149017</v>
       </c>
       <c r="C20" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="9" t="s">
-        <v>37</v>
-      </c>
       <c r="E20" s="10" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1369,13 +1372,13 @@
         <v>111424149018</v>
       </c>
       <c r="C21" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="D21" s="9" t="s">
-        <v>39</v>
-      </c>
       <c r="E21" s="10" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1386,13 +1389,13 @@
         <v>111424149019</v>
       </c>
       <c r="C22" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>41</v>
-      </c>
       <c r="E22" s="10" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1403,13 +1406,13 @@
         <v>111424149020</v>
       </c>
       <c r="C23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E23" s="12" t="s">
-        <v>118</v>
+      <c r="E23" s="11" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1420,13 +1423,13 @@
         <v>111424149021</v>
       </c>
       <c r="C24" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D24" s="9" t="s">
-        <v>45</v>
-      </c>
       <c r="E24" s="10" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1437,13 +1440,13 @@
         <v>111424149022</v>
       </c>
       <c r="C25" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D25" s="9" t="s">
-        <v>47</v>
-      </c>
       <c r="E25" s="10" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1454,13 +1457,13 @@
         <v>111424149023</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>121</v>
+        <v>142</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1471,13 +1474,13 @@
         <v>111424149024</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1488,13 +1491,13 @@
         <v>111424149025</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1505,13 +1508,13 @@
         <v>111424149026</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
@@ -1522,13 +1525,13 @@
         <v>111424149027</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1539,13 +1542,13 @@
         <v>111424149028</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1556,13 +1559,13 @@
         <v>111424149029</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1573,13 +1576,13 @@
         <v>111424149030</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1590,13 +1593,13 @@
         <v>111424149031</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="D34" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>146</v>
+        <v>62</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1607,13 +1610,13 @@
         <v>111424149032</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1624,13 +1627,13 @@
         <v>111424149033</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1641,13 +1644,13 @@
         <v>111424149035</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1658,13 +1661,13 @@
         <v>111424149036</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>135</v>
+        <v>144</v>
+      </c>
+      <c r="E38" s="11" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1675,13 +1678,13 @@
         <v>111424149037</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1692,13 +1695,13 @@
         <v>111424149038</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1709,13 +1712,13 @@
         <v>111424149039</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1726,13 +1729,13 @@
         <v>111424149040</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1743,13 +1746,13 @@
         <v>111424149041</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="E43" s="12" t="s">
-        <v>137</v>
+        <v>79</v>
+      </c>
+      <c r="E43" s="11" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1760,13 +1763,13 @@
         <v>111424149042</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E44" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="E44" s="11" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1777,13 +1780,13 @@
         <v>111424149043</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1794,13 +1797,13 @@
         <v>111424149044</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1811,13 +1814,13 @@
         <v>111424149045</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1828,13 +1831,13 @@
         <v>111424149046</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1845,13 +1848,13 @@
         <v>111424149047</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="E49" s="12" t="s">
-        <v>142</v>
+        <v>147</v>
+      </c>
+      <c r="E49" s="11" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1862,13 +1865,13 @@
         <v>111424149048</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1879,13 +1882,13 @@
         <v>111424149049</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -1904,6 +1907,7 @@
     <hyperlink ref="E49" r:id="rId12" xr:uid="{8864BC88-DF7F-4023-8D92-062CE90DB5A0}"/>
     <hyperlink ref="E44" r:id="rId13" xr:uid="{F46EEA24-0D18-4E74-BDE9-4051C32DF5EF}"/>
     <hyperlink ref="E34" r:id="rId14" xr:uid="{8C4C6B10-6941-4F8D-B442-F51E39EC1135}"/>
+    <hyperlink ref="E38" r:id="rId15" xr:uid="{CDA736F4-57B1-45A7-A195-7BEF66D5F38C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>